<commit_message>
Add press-release migration tooling for 6 additional categories
Generalize the article JCR generator with --category / --all / --rest
modes and per-category keywords + related-stories maps. Add <table>
support to the article parser (js + bundle) for financials earnings
tables. Include URL lists and import reports for financials,
innovation-driven, local-community-engagement, our-strategy, people-led,
and sustainable-services, plus a content/structural critique report
builder. Migration plan docs included.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article.report.xlsx
+++ b/tools/importer/reports/import-article.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1360" uniqueCount="690">
   <si>
     <t>_reportFile</t>
   </si>
@@ -536,6 +536,1542 @@
   </si>
   <si>
     <t>https://about.ups.com/us/en/newsroom/press-releases/customer-first/xin-ch-o-vietnam-country-welcomes-iconic-ups-browntail-for-first-time.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-move-to-virtual-annual-meeting-of-shareowners-for-2020.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-move-to-virtual-annual-meeting-of-shareowners-for-2020</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:40:15.824Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-announces-move-to-virtual-annual-meeting-of-shareowners-for-2020.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-2q2021.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-2q2021</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:40:08.283Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/UPS-announces-quarterly-dividend-2Q2021.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-and-5-billion-share-repurchase.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-and-5-billion-share-repurchase</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:40:48.098Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-and--5-billion-share-repurchase.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q1-2022.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q1-2022</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:40:55.776Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q1-2022.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q1-2025.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q1-2025</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:39:44.629Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/-ups-announces-quarterly-dividend-q1-2025.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q2-2022.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q2-2022</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:41:04.084Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q2-2022.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q2-2024.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q2-2024</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:40:24.201Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend---q2-2024.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q22023.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q22023</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:41:12.467Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q22023.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q3-2022.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q3-2022</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:41:19.853Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q3-2022.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q3-2023.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q3-2023</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:41:28.844Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q3-2023.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q3-2024.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q3-2024</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:40:32.869Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend---q3-2024.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q4-2024.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend-q4-2024</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:40:40.668Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend---q4-2024.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:41:35.849Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend0.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend0</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:41:42.759Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend0.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend1.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend1</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:41:49.651Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend1.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend2.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend2</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:41:57.238Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend2.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend3.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend3</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:42:04.514Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend3.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend4.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend4</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:42:13.026Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend4.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend5.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend5</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:42:20.526Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-announces-quarterly-dividend5.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-strategic-initiatives-and-three-year-financial-tar.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-strategic-initiatives-and-three-year-financial-tar</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:42:28.550Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-announces-strategic-initiatives-and-three-year-financial-tar.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-strategic-priorities-three-year-financial-targets.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-announces-strategic-priorities-three-year-financial-targets</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:42:35.385Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-announces-strategic-priorities--three-year-financial-targets.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-board-increases-quarterly-dividend-1.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-board-increases-quarterly-dividend-1</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:42:41.833Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-board-increases-quarterly-dividend-1.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-board-increases-quarterly-dividend.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-board-increases-quarterly-dividend</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:42:48.721Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-board-increases-quarterly-dividend.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-delivers-1q-2018-eps-of-1-55-up-17.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-delivers-1q-2018-eps-of-1-55-up-17</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:42:57.078Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-delivers-1q-2018-eps-of-1-55-up-17-.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-holds-shareowners-meeting-elects-board-members.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-holds-shareowners-meeting-elects-board-members</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:43:04.303Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-holds-shareowners-meeting-elects-board-members.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-1q-2020-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-1q-2020-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:43:12.506Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-1q-2020-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-1q-2021-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-1q-2021-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:43:20.174Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-1q-2021-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-1q-2022-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-1q-2022-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:43:27.816Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-1q-2022-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-1q-2023-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-1q-2023-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:43:35.071Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-1q-2023-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-1q-2024-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-1q-2024-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:43:42.657Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-1q-2024-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-1q-2025-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-1q-2025-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:43:51.082Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-1q-2025-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-1q-2026-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-1q-2026-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:43:59.185Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-1q-2026-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-2q-2020-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-2q-2020-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:44:06.467Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-2q-2020-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-2q-2022-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-2q-2022-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:44:15.112Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-2q-2022-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-2q-2023-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-2q-2023-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:44:22.626Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-2q-2023-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-2q-2024-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-2q-2024-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:44:30.330Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-2q-2024-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-2q-2025-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-2q-2025-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:44:38.097Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-2q-2025-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-3q-2019-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-3q-2019-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:44:46.108Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-3q-2019-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-3q-2020-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-3q-2020-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:44:53.216Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-3q-2020-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-3q-2022-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-3q-2022-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:45:00.486Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-3q-2022-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-3q-2023-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-3q-2023-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:39:52.862Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/UPS-RELEASES-3Q-2023-EARNINGS.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-3q-2024-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-3q-2024-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:45:07.646Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-3q-2024-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-3q-2025-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-3q-2025-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:45:15.647Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-3q-2025-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-4q-2019-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-4q-2019-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:45:23.528Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-4q-2019-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-4q-2020-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-4q-2020-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:45:30.738Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-4q-2020-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-4q-2022-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-4q-2022-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:45:39.927Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-4q-2022-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-4q-2023-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-4q-2023-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:45:47.559Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-4q-2023-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-4q-2024-earnings-and-provides-2025-guidance.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-4q-2024-earnings-and-provides-2025-guidance</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:45:56.155Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-4q-2024-earnings-and-provides-2025-guidance.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-4q-2025-earnings-and-provides-2026-guidance.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-4q-2025-earnings-and-provides-2026-guidance</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:46:04.917Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-4q-2025-earnings-and-provides-2026-guidance.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-q1-2021-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-q1-2021-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:46:13.330Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-q1-2021-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-q3-2021-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-q3-2021-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:46:21.150Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-q3-2021-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-q4-2021-earnings.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-releases-q4-2021-earnings</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:46:29.331Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-releases-q4-2021-earnings.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-first-quarter-2021-results.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-first-quarter-2021-results</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:46:36.442Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-first-quarter-2021-results.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-first-quarter-2022-results.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-first-quarter-2022-results</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:46:44.427Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-first-quarter-2022-results.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-first-quarter-2024-results.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-first-quarter-2024-results</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:46:50.857Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-first-quarter-2024-results.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-first-quarter-2025-results-on-tuesday-april-29.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-first-quarter-2025-results-on-tuesday-april-29</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:46:58.912Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-first-quarter-2025-results-on-tuesday--april-29--.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-first-quarter-2026-results-on-tuesday-april-28.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-first-quarter-2026-results-on-tuesday-april-28</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:47:07.559Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-first-quarter-2026-results-on-tuesday--april-28--.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-first-quarter-results-on-tuesday-april-28-2020.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-first-quarter-results-on-tuesday-april-28-2020</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:47:16.211Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-first-quarter-results-on-tuesday-april-28-2020.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2020-results-on-tuesday-feb-2-2021.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2020-results-on-tuesday-feb-2-2021</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:47:25.529Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2020-results-on-tuesday-feb-2-2021.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2021-results.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2021-results</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:47:32.576Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2021-results.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2022-results.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2022-results</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:47:39.712Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2022-results.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2022-results0.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2022-results0</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:47:47.560Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2022-results0.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2023-results.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2023-results</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:40:00.015Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/UPS-To-Release-Fourth-Quarter-2023-Results.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2024-results-on-thursday-january.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2024-results-on-thursday-january</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:47:53.977Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2024-results-on-thursday--january-.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2025-results-on-tuesday-january-2.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2025-results-on-tuesday-january-2</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:48:02.069Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-2025-results-on-tuesday--january-2.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-results-on-thursday-january-30-2020.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-results-on-thursday-january-30-2020</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:48:09.660Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-fourth-quarter-results-on-thursday-january-30-2020.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-second-quarter-2021-results.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-second-quarter-2021-results</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:48:15.928Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-second-quarter-2021-results.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-second-quarter-2022-results.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-second-quarter-2022-results</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:48:23.497Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-second-quarter-2022-results.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-second-quarter-2024-results-on-tuesday-july-23-20.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-second-quarter-2024-results-on-tuesday-july-23-20</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:48:30.593Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-second-quarter-2024-results-on-tuesday-july-23-20.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-second-quarter-2025-results-on-tuesday-july-29.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-second-quarter-2025-results-on-tuesday-july-29</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:48:37.741Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-second-quarter-2025-results-on-tuesday--july-29--.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-second-quarter-results-on-thursday-july-30-2020.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-second-quarter-results-on-thursday-july-30-2020</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:48:44.553Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-second-quarter-results-on-thursday-july-30-2020.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-third-quarter-2022-results.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-third-quarter-2022-results</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:48:52.077Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-third-quarter-2022-results.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-third-quarter-2023-results.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/financials/ups-to-release-third-quarter-2023-results</t>
+  </si>
+  <si>
+    <t>2026-07-24T11:48:58.586Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/financials/ups-to-release-third-quarter-2023-results.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/innovation-driven/coyote-logistics-launches-dynamic-route-optimization-to-enhance-supply-chain-efficiency.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/innovation-driven/coyote-logistics-launches-dynamic-route-optimization-to-enhance-supply-chain-efficiency</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:30:18.426Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/innovation-driven/coyote-logistics-launches-dynamic-route-optimization-to-enhance-supply-chain-efficiency.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/innovation-driven/new-chief-digital-and-technology-officer.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/innovation-driven/new-chief-digital-and-technology-officer</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:30:26.846Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/innovation-driven/new-chief-digital-and-technology-officer.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/innovation-driven/ups-deploys-purpose-built-navigation-for-ups-service-personnel.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/innovation-driven/ups-deploys-purpose-built-navigation-for-ups-service-personnel</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:30:35.352Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/innovation-driven/ups-deploys-purpose-built-navigation-for-ups-service-personnel.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/innovation-driven/ups-flight-forward-adds-new-aircraft.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/innovation-driven/ups-flight-forward-adds-new-aircraft</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:30:42.678Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/innovation-driven/ups-flight-forward-adds-new-aircraft.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/innovation-driven/ups-strengthens-network-capabilities-and-employee-experience-th.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/innovation-driven/ups-strengthens-network-capabilities-and-employee-experience-th</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:30:50.420Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/innovation-driven/ups-strengthens-network-capabilities-and-employee-experience--th.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/innovation-driven/ups-to-test-gaussin-autonomous-enabled-ev-s-to-move-trailers-at-its-london-hub.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/innovation-driven/ups-to-test-gaussin-autonomous-enabled-ev-s-to-move-trailers-at-its-london-hub</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:30:57.358Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/innovation-driven/ups-to-test-gaussin-autonomous-enabled-ev-s-to-move-trailers-at-its-london-hub.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/local-community-engagement/allocates-15m-to-fight-against-coronavirus.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/local-community-engagement/allocates-15m-to-fight-against-coronavirus</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:55:54.558Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/local-community-engagement/allocates-15m-to-fight-against-coronavirus.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/local-community-engagement/combat-novel-coronavirus-around-the-world.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/local-community-engagement/combat-novel-coronavirus-around-the-world</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:56:01.735Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/local-community-engagement/combat-novel-coronavirus-around-the-world.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/local-community-engagement/mobilizes-global-relief-in-australia-puerto-rico-philippines.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/local-community-engagement/mobilizes-global-relief-in-australia-puerto-rico-philippines</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:56:09.528Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/local-community-engagement/mobilizes-global-relief-in-australia-puerto-rico-philippines.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/local-community-engagement/never-forget-upsers-pay-tribute-to-9-11-heroes.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/local-community-engagement/never-forget-upsers-pay-tribute-to-9-11-heroes</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:56:17.978Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/local-community-engagement/never-forget-upsers-pay-tribute-to-9-11-heroes.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/local-community-engagement/ups-donates-nearly-500-000-in-new-funding-to-kentucky-indiana-ohio-nonprofits-university-of-louisville-for-coronavirus-relief.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/local-community-engagement/ups-donates-nearly-500-000-in-new-funding-to-kentucky-indiana-ohio-nonprofits-university-of-louisville-for-coronavirus-relief</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:56:24.895Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/local-community-engagement/ups-donates-nearly-500-000-in-new-funding-to-kentucky-indiana-ohio-nonprofits-university-of-louisville-for-coronavirus-relief.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/local-community-engagement/ups-expedites-global-deliveries-of-qiagen-coronavirus-testing-kits.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/local-community-engagement/ups-expedites-global-deliveries-of-qiagen-coronavirus-testing-kits</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:56:32.466Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/local-community-engagement/ups-expedites-global-deliveries-of-qiagen-coronavirus-testing-kits.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/local-community-engagement/ups-impact-summit.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/local-community-engagement/ups-impact-summit</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:56:40.001Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/local-community-engagement/ups-impact-summit.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/local-community-engagement/ups-supporting-university-of-louisville-manufacturing-of-face-shields.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/local-community-engagement/ups-supporting-university-of-louisville-manufacturing-of-face-shields</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:56:47.116Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/local-community-engagement/ups-supporting-university-of-louisville-manufacturing-of-face-shields.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/2023-ups-impact-summit.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/2023-ups-impact-summit</t>
+  </si>
+  <si>
+    <t>2026-07-24T13:12:20.654Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/our-strategy/2023-ups-impact-summit.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/ups-acquires-andlauer-healthcare-group-for-1-6-billion-acceler.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/ups-acquires-andlauer-healthcare-group-for-1-6-billion-acceler</t>
+  </si>
+  <si>
+    <t>2026-07-24T13:12:27.543Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/our-strategy/ups-acquires-andlauer-healthcare-group-for--1-6-billion--acceler.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/ups-and-international-brotherhood-of-teamsters-reach-handshake-agreement-for-new-national-master-agreement.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/ups-and-international-brotherhood-of-teamsters-reach-handshake-agreement-for-new-national-master-agreement</t>
+  </si>
+  <si>
+    <t>2026-07-24T13:12:36.496Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/our-strategy/ups-and-international-brotherhood-of-teamsters-reach-handshake-agreement-for-new-national-master-agreement.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/ups-and-international-brotherhood-of-teamsters-reach-tentative-new-national-master-ups-freight-agreement.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/ups-and-international-brotherhood-of-teamsters-reach-tentative-new-national-master-ups-freight-agreement</t>
+  </si>
+  <si>
+    <t>2026-07-24T13:12:43.816Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/our-strategy/ups-and-international-brotherhood-of-teamsters-reach-tentative-new-national-master-ups-freight-agreement.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/ups-announces-agreement-to-sell-ups-freight-to-tfi-international.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/ups-announces-agreement-to-sell-ups-freight-to-tfi-international</t>
+  </si>
+  <si>
+    <t>2026-07-24T13:12:50.827Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/our-strategy/ups-announces-agreement-to-sell-ups-freight-to-tfi-international.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/ups-announces-sale-of-coyote-logistics-to-rxo-inc.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/ups-announces-sale-of-coyote-logistics-to-rxo-inc</t>
+  </si>
+  <si>
+    <t>2026-07-24T13:12:59.721Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/our-strategy/ups-announces-sale-of-coyote-logistics-to-rxo--inc-.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/ups-bolsters-healthcare-logistics-capabilities-with-cold-chain-a.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/ups-bolsters-healthcare-logistics-capabilities-with-cold-chain-a</t>
+  </si>
+  <si>
+    <t>2026-07-24T13:13:06.479Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/our-strategy/ups-bolsters-healthcare-logistics-capabilities-with-cold-chain-a.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/ups-completes-acquisitions-of-healthcare-cold-chain-logistics-pr.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/ups-completes-acquisitions-of-healthcare-cold-chain-logistics-pr</t>
+  </si>
+  <si>
+    <t>2026-07-24T13:13:15.271Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/our-strategy/ups-completes-acquisitions-of-healthcare-cold-chain-logistics-pr.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/ups-to-acquire-andlauer-healthcare-group-for-1-6-billion-stren.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/ups-to-acquire-andlauer-healthcare-group-for-1-6-billion-stren</t>
+  </si>
+  <si>
+    <t>2026-07-24T13:13:21.559Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/our-strategy/ups-to-acquire-andlauer-healthcare-group-for--1-6-billion--stren.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/ups-to-acquire-estafeta-providing-powerful-global-logistics-sol.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/our-strategy/ups-to-acquire-estafeta-providing-powerful-global-logistics-sol</t>
+  </si>
+  <si>
+    <t>2026-07-24T13:13:28.488Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/our-strategy/ups-to-acquire-estafeta--providing-powerful-global-logistics-sol.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/circle-of-honor-2022-announcement.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/circle-of-honor-2022-announcement</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:21:12.242Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/circle-of-honor-2022-announcement.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/iconic-ups-brown-delivery-vehicles-receive-personal-update.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/iconic-ups-brown-delivery-vehicles-receive-personal-update</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:21:19.620Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/iconic-ups-brown-delivery-vehicles-receive-personal-update.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/teamsters-approve-strike-authorization.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/teamsters-approve-strike-authorization</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:21:26.577Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/teamsters-approve-strike-authorization.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-announces-changes-to-board-of-directors.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-announces-changes-to-board-of-directors</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:21:40.482Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-announces-changes-to-board-of-directors.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-announces-executive-leadership-team-changes.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-announces-executive-leadership-team-changes</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:21:48.055Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-announces-executive-leadership-team-changes.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-announces-organizational-realignment.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-announces-organizational-realignment</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:21:54.752Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-announces-organizational-realignment.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-appoints-brian-dykes-as-chief-financial-officer.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-appoints-brian-dykes-as-chief-financial-officer</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:22:02.744Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-appoints-brian-dykes-as-chief-financial-officer.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-appoints-eva-boratto-and-wayne-hewett-to-board-of-directors.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-appoints-eva-boratto-and-wayne-hewett-to-board-of-directors</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:22:10.029Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-appoints-eva-boratto-and-wayne-hewett-to-board-of-directors.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-appoints-john-morikis-to-board-of-directors.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-appoints-john-morikis-to-board-of-directors</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:22:16.956Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-appoints-john-morikis-to-board-of-directors.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-appoints-kevin-clark-to-board-of-directors.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-appoints-kevin-clark-to-board-of-directors</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:22:23.517Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-appoints-kevin-clark-to-board-of-directors.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-asks-job-seekers-to-picture-yourself-in-ups-brown.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-asks-job-seekers-to-picture-yourself-in-ups-brown</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:22:31.084Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-asks-job-seekers-to--picture-yourself-in-ups-brown-.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-board-appoints-carol-tom-as-ceo-david-abney-to-be-executive-chairman.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-board-appoints-carol-tom-as-ceo-david-abney-to-be-executive-chairman</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:22:37.665Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-board-appoints-carol-tom-as-ceo-david-abney-to-be-executive-chairman.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-chief-financial-officer-brian-newman-to-depart.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-chief-financial-officer-brian-newman-to-depart</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:21:05.202Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/-ups-chief-financial-officer-brian-newman-to-depart.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-encouraged-that-the-teamsters-will-continue-forward-progress.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-encouraged-that-the-teamsters-will-continue-forward-progress</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:22:44.856Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-encouraged-that-the-teamsters-will-continue-forward-progress.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-encourages-teamsters-to-return-to-the-negotiations-table.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-encourages-teamsters-to-return-to-the-negotiations-table</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:22:52.906Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-encourages-teamsters-to-return-to-the-negotiations-table.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-inducts-1-412-of-its-safest-drivers-into-circle-of-honor.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-inducts-1-412-of-its-safest-drivers-into-circle-of-honor</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:22:59.742Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-inducts-1-412-of-its-safest-drivers-into-circle-of-honor.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-invests-millions-in-advanced-training-for-on-the-road-driver.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-invests-millions-in-advanced-training-for-on-the-road-driver</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:23:05.418Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-invests-millions-in-advanced-training-for-on-the-road-driver.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-names-angela-hwang-to-board-of-directors.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-names-angela-hwang-to-board-of-directors</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:23:13.654Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-names-angela-hwang-to-board-of-directors.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-promotes-laura-lane-to-chief-corporate-affairs-and-communications-officer.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-promotes-laura-lane-to-chief-corporate-affairs-and-communications-officer</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:23:21.305Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-promotes-laura-lane-to-chief-corporate-affairs-and-communications-officer.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-recruits-100-000-seasonal-workers-for-the-2023-holiday-seaso.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-recruits-100-000-seasonal-workers-for-the-2023-holiday-seaso</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:23:27.905Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-recruits-100-000-seasonal-workers-for-the-2023-holiday-seaso.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-releases-first-jobs-and-opportunity-report.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-releases-first-jobs-and-opportunity-report</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:23:34.764Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-releases-first-jobs-and-opportunity-report.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-responds-to-latest-action-from-the-teamsters.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-responds-to-latest-action-from-the-teamsters</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:23:42.683Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-responds-to-latest-action-from-the-teamsters.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-starts-business-continuity-training.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-starts-business-continuity-training</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:23:50.828Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-starts-business-continuity-training.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-statement-agreement-with-teamsters-on-heat-safety.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-statement-agreement-with-teamsters-on-heat-safety</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:23:57.980Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-statement-agreement-with-teamsters-on-heat-safety.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-statement-on-teamster-negotiations.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-statement-on-teamster-negotiations</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:24:05.726Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-statement-on-teamster-negotiations.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-teamsters-negotiations-to-resume-next-week.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-teamsters-negotiations-to-resume-next-week</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:21:33.942Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups--teamsters-negotiations-to-resume-next-week.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-teamsters-reach-agreement-in-labor-negotiations.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-teamsters-reach-agreement-in-labor-negotiations</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:24:13.486Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-teamsters-reach-agreement-in-labor-negotiations.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-to-hire-over-100-000.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/people-led/ups-to-hire-over-100-000</t>
+  </si>
+  <si>
+    <t>2026-07-24T12:24:20.397Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/people-led/ups-to-hire-over-100-000-.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/sustainable-services/news-hurricane-laura-relief-efforts-supported-by-ups-strategy-of-preparedness.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/sustainable-services/news-hurricane-laura-relief-efforts-supported-by-ups-strategy-of-preparedness</t>
+  </si>
+  <si>
+    <t>2026-07-24T13:17:01.149Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/sustainable-services/news-hurricane-laura-relief-efforts-supported-by-ups-strategy-of-preparedness.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/sustainable-services/ups-appoints-nikki-clifton-to-lead-the-ups-foundation-announces-retirement-of-ed-martinez-after-44-years-of-distinguished-service.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/sustainable-services/ups-appoints-nikki-clifton-to-lead-the-ups-foundation-announces-retirement-of-ed-martinez-after-44-years-of-distinguished-service</t>
+  </si>
+  <si>
+    <t>2026-07-24T13:17:09.257Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/sustainable-services/ups-appoints-nikki-clifton-to-lead-the-ups-foundation-announces-retirement-of-ed-martinez-after-44-years-of-distinguished-service.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/sustainable-services/ups-invests-in-arrival-accelerates-fleet-electrification-with-order-of-10-000-electric-delivery-vehicles.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/press-releases/sustainable-services/ups-invests-in-arrival-accelerates-fleet-electrification-with-order-of-10-000-electric-delivery-vehicles</t>
+  </si>
+  <si>
+    <t>2026-07-24T13:17:16.999Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/press-releases/sustainable-services/ups-invests-in-arrival-accelerates-fleet-electrification-with-order-of-10-000-electric-delivery-vehicles.html</t>
   </si>
   <si>
     <t>content/language-masters/en/newsroom/press-releases/customer-first/ups-extends-complex-healthcare-logistics-lead-with-48-million-i.report.json</t>
@@ -933,7 +2469,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H170"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -2032,6 +3568,3334 @@
         <v>21</v>
       </c>
       <c r="H42" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>179</v>
+      </c>
+      <c r="B43" t="s">
+        <v>17</v>
+      </c>
+      <c r="C43" t="s">
+        <v>180</v>
+      </c>
+      <c r="D43" t="s">
+        <v>11</v>
+      </c>
+      <c r="E43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F43" t="s">
+        <v>181</v>
+      </c>
+      <c r="G43" t="s">
+        <v>21</v>
+      </c>
+      <c r="H43" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>183</v>
+      </c>
+      <c r="B44" t="s">
+        <v>17</v>
+      </c>
+      <c r="C44" t="s">
+        <v>184</v>
+      </c>
+      <c r="D44" t="s">
+        <v>11</v>
+      </c>
+      <c r="E44" t="s">
+        <v>19</v>
+      </c>
+      <c r="F44" t="s">
+        <v>185</v>
+      </c>
+      <c r="G44" t="s">
+        <v>21</v>
+      </c>
+      <c r="H44" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>187</v>
+      </c>
+      <c r="B45" t="s">
+        <v>17</v>
+      </c>
+      <c r="C45" t="s">
+        <v>188</v>
+      </c>
+      <c r="D45" t="s">
+        <v>11</v>
+      </c>
+      <c r="E45" t="s">
+        <v>19</v>
+      </c>
+      <c r="F45" t="s">
+        <v>189</v>
+      </c>
+      <c r="G45" t="s">
+        <v>21</v>
+      </c>
+      <c r="H45" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>191</v>
+      </c>
+      <c r="B46" t="s">
+        <v>17</v>
+      </c>
+      <c r="C46" t="s">
+        <v>192</v>
+      </c>
+      <c r="D46" t="s">
+        <v>11</v>
+      </c>
+      <c r="E46" t="s">
+        <v>19</v>
+      </c>
+      <c r="F46" t="s">
+        <v>193</v>
+      </c>
+      <c r="G46" t="s">
+        <v>21</v>
+      </c>
+      <c r="H46" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>195</v>
+      </c>
+      <c r="B47" t="s">
+        <v>17</v>
+      </c>
+      <c r="C47" t="s">
+        <v>196</v>
+      </c>
+      <c r="D47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" t="s">
+        <v>19</v>
+      </c>
+      <c r="F47" t="s">
+        <v>197</v>
+      </c>
+      <c r="G47" t="s">
+        <v>21</v>
+      </c>
+      <c r="H47" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>199</v>
+      </c>
+      <c r="B48" t="s">
+        <v>17</v>
+      </c>
+      <c r="C48" t="s">
+        <v>200</v>
+      </c>
+      <c r="D48" t="s">
+        <v>11</v>
+      </c>
+      <c r="E48" t="s">
+        <v>19</v>
+      </c>
+      <c r="F48" t="s">
+        <v>201</v>
+      </c>
+      <c r="G48" t="s">
+        <v>21</v>
+      </c>
+      <c r="H48" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>203</v>
+      </c>
+      <c r="B49" t="s">
+        <v>17</v>
+      </c>
+      <c r="C49" t="s">
+        <v>204</v>
+      </c>
+      <c r="D49" t="s">
+        <v>11</v>
+      </c>
+      <c r="E49" t="s">
+        <v>19</v>
+      </c>
+      <c r="F49" t="s">
+        <v>205</v>
+      </c>
+      <c r="G49" t="s">
+        <v>21</v>
+      </c>
+      <c r="H49" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>207</v>
+      </c>
+      <c r="B50" t="s">
+        <v>17</v>
+      </c>
+      <c r="C50" t="s">
+        <v>208</v>
+      </c>
+      <c r="D50" t="s">
+        <v>11</v>
+      </c>
+      <c r="E50" t="s">
+        <v>19</v>
+      </c>
+      <c r="F50" t="s">
+        <v>209</v>
+      </c>
+      <c r="G50" t="s">
+        <v>21</v>
+      </c>
+      <c r="H50" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>211</v>
+      </c>
+      <c r="B51" t="s">
+        <v>17</v>
+      </c>
+      <c r="C51" t="s">
+        <v>212</v>
+      </c>
+      <c r="D51" t="s">
+        <v>11</v>
+      </c>
+      <c r="E51" t="s">
+        <v>19</v>
+      </c>
+      <c r="F51" t="s">
+        <v>213</v>
+      </c>
+      <c r="G51" t="s">
+        <v>21</v>
+      </c>
+      <c r="H51" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>215</v>
+      </c>
+      <c r="B52" t="s">
+        <v>17</v>
+      </c>
+      <c r="C52" t="s">
+        <v>216</v>
+      </c>
+      <c r="D52" t="s">
+        <v>11</v>
+      </c>
+      <c r="E52" t="s">
+        <v>19</v>
+      </c>
+      <c r="F52" t="s">
+        <v>217</v>
+      </c>
+      <c r="G52" t="s">
+        <v>21</v>
+      </c>
+      <c r="H52" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>219</v>
+      </c>
+      <c r="B53" t="s">
+        <v>17</v>
+      </c>
+      <c r="C53" t="s">
+        <v>220</v>
+      </c>
+      <c r="D53" t="s">
+        <v>11</v>
+      </c>
+      <c r="E53" t="s">
+        <v>19</v>
+      </c>
+      <c r="F53" t="s">
+        <v>221</v>
+      </c>
+      <c r="G53" t="s">
+        <v>21</v>
+      </c>
+      <c r="H53" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>223</v>
+      </c>
+      <c r="B54" t="s">
+        <v>17</v>
+      </c>
+      <c r="C54" t="s">
+        <v>224</v>
+      </c>
+      <c r="D54" t="s">
+        <v>11</v>
+      </c>
+      <c r="E54" t="s">
+        <v>19</v>
+      </c>
+      <c r="F54" t="s">
+        <v>225</v>
+      </c>
+      <c r="G54" t="s">
+        <v>21</v>
+      </c>
+      <c r="H54" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>227</v>
+      </c>
+      <c r="B55" t="s">
+        <v>17</v>
+      </c>
+      <c r="C55" t="s">
+        <v>228</v>
+      </c>
+      <c r="D55" t="s">
+        <v>11</v>
+      </c>
+      <c r="E55" t="s">
+        <v>19</v>
+      </c>
+      <c r="F55" t="s">
+        <v>229</v>
+      </c>
+      <c r="G55" t="s">
+        <v>21</v>
+      </c>
+      <c r="H55" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>231</v>
+      </c>
+      <c r="B56" t="s">
+        <v>17</v>
+      </c>
+      <c r="C56" t="s">
+        <v>232</v>
+      </c>
+      <c r="D56" t="s">
+        <v>11</v>
+      </c>
+      <c r="E56" t="s">
+        <v>19</v>
+      </c>
+      <c r="F56" t="s">
+        <v>233</v>
+      </c>
+      <c r="G56" t="s">
+        <v>21</v>
+      </c>
+      <c r="H56" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>235</v>
+      </c>
+      <c r="B57" t="s">
+        <v>17</v>
+      </c>
+      <c r="C57" t="s">
+        <v>236</v>
+      </c>
+      <c r="D57" t="s">
+        <v>11</v>
+      </c>
+      <c r="E57" t="s">
+        <v>19</v>
+      </c>
+      <c r="F57" t="s">
+        <v>237</v>
+      </c>
+      <c r="G57" t="s">
+        <v>21</v>
+      </c>
+      <c r="H57" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>239</v>
+      </c>
+      <c r="B58" t="s">
+        <v>17</v>
+      </c>
+      <c r="C58" t="s">
+        <v>240</v>
+      </c>
+      <c r="D58" t="s">
+        <v>11</v>
+      </c>
+      <c r="E58" t="s">
+        <v>19</v>
+      </c>
+      <c r="F58" t="s">
+        <v>241</v>
+      </c>
+      <c r="G58" t="s">
+        <v>21</v>
+      </c>
+      <c r="H58" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>243</v>
+      </c>
+      <c r="B59" t="s">
+        <v>17</v>
+      </c>
+      <c r="C59" t="s">
+        <v>244</v>
+      </c>
+      <c r="D59" t="s">
+        <v>11</v>
+      </c>
+      <c r="E59" t="s">
+        <v>19</v>
+      </c>
+      <c r="F59" t="s">
+        <v>245</v>
+      </c>
+      <c r="G59" t="s">
+        <v>21</v>
+      </c>
+      <c r="H59" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>247</v>
+      </c>
+      <c r="B60" t="s">
+        <v>17</v>
+      </c>
+      <c r="C60" t="s">
+        <v>248</v>
+      </c>
+      <c r="D60" t="s">
+        <v>11</v>
+      </c>
+      <c r="E60" t="s">
+        <v>19</v>
+      </c>
+      <c r="F60" t="s">
+        <v>249</v>
+      </c>
+      <c r="G60" t="s">
+        <v>21</v>
+      </c>
+      <c r="H60" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>251</v>
+      </c>
+      <c r="B61" t="s">
+        <v>17</v>
+      </c>
+      <c r="C61" t="s">
+        <v>252</v>
+      </c>
+      <c r="D61" t="s">
+        <v>11</v>
+      </c>
+      <c r="E61" t="s">
+        <v>19</v>
+      </c>
+      <c r="F61" t="s">
+        <v>253</v>
+      </c>
+      <c r="G61" t="s">
+        <v>21</v>
+      </c>
+      <c r="H61" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>255</v>
+      </c>
+      <c r="B62" t="s">
+        <v>17</v>
+      </c>
+      <c r="C62" t="s">
+        <v>256</v>
+      </c>
+      <c r="D62" t="s">
+        <v>11</v>
+      </c>
+      <c r="E62" t="s">
+        <v>19</v>
+      </c>
+      <c r="F62" t="s">
+        <v>257</v>
+      </c>
+      <c r="G62" t="s">
+        <v>21</v>
+      </c>
+      <c r="H62" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>259</v>
+      </c>
+      <c r="B63" t="s">
+        <v>17</v>
+      </c>
+      <c r="C63" t="s">
+        <v>260</v>
+      </c>
+      <c r="D63" t="s">
+        <v>11</v>
+      </c>
+      <c r="E63" t="s">
+        <v>19</v>
+      </c>
+      <c r="F63" t="s">
+        <v>261</v>
+      </c>
+      <c r="G63" t="s">
+        <v>21</v>
+      </c>
+      <c r="H63" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>263</v>
+      </c>
+      <c r="B64" t="s">
+        <v>17</v>
+      </c>
+      <c r="C64" t="s">
+        <v>264</v>
+      </c>
+      <c r="D64" t="s">
+        <v>11</v>
+      </c>
+      <c r="E64" t="s">
+        <v>19</v>
+      </c>
+      <c r="F64" t="s">
+        <v>265</v>
+      </c>
+      <c r="G64" t="s">
+        <v>21</v>
+      </c>
+      <c r="H64" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>267</v>
+      </c>
+      <c r="B65" t="s">
+        <v>17</v>
+      </c>
+      <c r="C65" t="s">
+        <v>268</v>
+      </c>
+      <c r="D65" t="s">
+        <v>11</v>
+      </c>
+      <c r="E65" t="s">
+        <v>19</v>
+      </c>
+      <c r="F65" t="s">
+        <v>269</v>
+      </c>
+      <c r="G65" t="s">
+        <v>21</v>
+      </c>
+      <c r="H65" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>271</v>
+      </c>
+      <c r="B66" t="s">
+        <v>17</v>
+      </c>
+      <c r="C66" t="s">
+        <v>272</v>
+      </c>
+      <c r="D66" t="s">
+        <v>11</v>
+      </c>
+      <c r="E66" t="s">
+        <v>19</v>
+      </c>
+      <c r="F66" t="s">
+        <v>273</v>
+      </c>
+      <c r="G66" t="s">
+        <v>21</v>
+      </c>
+      <c r="H66" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>275</v>
+      </c>
+      <c r="B67" t="s">
+        <v>17</v>
+      </c>
+      <c r="C67" t="s">
+        <v>276</v>
+      </c>
+      <c r="D67" t="s">
+        <v>11</v>
+      </c>
+      <c r="E67" t="s">
+        <v>19</v>
+      </c>
+      <c r="F67" t="s">
+        <v>277</v>
+      </c>
+      <c r="G67" t="s">
+        <v>21</v>
+      </c>
+      <c r="H67" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>279</v>
+      </c>
+      <c r="B68" t="s">
+        <v>17</v>
+      </c>
+      <c r="C68" t="s">
+        <v>280</v>
+      </c>
+      <c r="D68" t="s">
+        <v>11</v>
+      </c>
+      <c r="E68" t="s">
+        <v>19</v>
+      </c>
+      <c r="F68" t="s">
+        <v>281</v>
+      </c>
+      <c r="G68" t="s">
+        <v>21</v>
+      </c>
+      <c r="H68" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>283</v>
+      </c>
+      <c r="B69" t="s">
+        <v>17</v>
+      </c>
+      <c r="C69" t="s">
+        <v>284</v>
+      </c>
+      <c r="D69" t="s">
+        <v>11</v>
+      </c>
+      <c r="E69" t="s">
+        <v>19</v>
+      </c>
+      <c r="F69" t="s">
+        <v>285</v>
+      </c>
+      <c r="G69" t="s">
+        <v>21</v>
+      </c>
+      <c r="H69" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>287</v>
+      </c>
+      <c r="B70" t="s">
+        <v>17</v>
+      </c>
+      <c r="C70" t="s">
+        <v>288</v>
+      </c>
+      <c r="D70" t="s">
+        <v>11</v>
+      </c>
+      <c r="E70" t="s">
+        <v>19</v>
+      </c>
+      <c r="F70" t="s">
+        <v>289</v>
+      </c>
+      <c r="G70" t="s">
+        <v>21</v>
+      </c>
+      <c r="H70" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>291</v>
+      </c>
+      <c r="B71" t="s">
+        <v>17</v>
+      </c>
+      <c r="C71" t="s">
+        <v>292</v>
+      </c>
+      <c r="D71" t="s">
+        <v>11</v>
+      </c>
+      <c r="E71" t="s">
+        <v>19</v>
+      </c>
+      <c r="F71" t="s">
+        <v>293</v>
+      </c>
+      <c r="G71" t="s">
+        <v>21</v>
+      </c>
+      <c r="H71" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>295</v>
+      </c>
+      <c r="B72" t="s">
+        <v>17</v>
+      </c>
+      <c r="C72" t="s">
+        <v>296</v>
+      </c>
+      <c r="D72" t="s">
+        <v>11</v>
+      </c>
+      <c r="E72" t="s">
+        <v>19</v>
+      </c>
+      <c r="F72" t="s">
+        <v>297</v>
+      </c>
+      <c r="G72" t="s">
+        <v>21</v>
+      </c>
+      <c r="H72" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>299</v>
+      </c>
+      <c r="B73" t="s">
+        <v>17</v>
+      </c>
+      <c r="C73" t="s">
+        <v>300</v>
+      </c>
+      <c r="D73" t="s">
+        <v>11</v>
+      </c>
+      <c r="E73" t="s">
+        <v>19</v>
+      </c>
+      <c r="F73" t="s">
+        <v>301</v>
+      </c>
+      <c r="G73" t="s">
+        <v>21</v>
+      </c>
+      <c r="H73" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>303</v>
+      </c>
+      <c r="B74" t="s">
+        <v>17</v>
+      </c>
+      <c r="C74" t="s">
+        <v>304</v>
+      </c>
+      <c r="D74" t="s">
+        <v>11</v>
+      </c>
+      <c r="E74" t="s">
+        <v>19</v>
+      </c>
+      <c r="F74" t="s">
+        <v>305</v>
+      </c>
+      <c r="G74" t="s">
+        <v>21</v>
+      </c>
+      <c r="H74" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>307</v>
+      </c>
+      <c r="B75" t="s">
+        <v>17</v>
+      </c>
+      <c r="C75" t="s">
+        <v>308</v>
+      </c>
+      <c r="D75" t="s">
+        <v>11</v>
+      </c>
+      <c r="E75" t="s">
+        <v>19</v>
+      </c>
+      <c r="F75" t="s">
+        <v>309</v>
+      </c>
+      <c r="G75" t="s">
+        <v>21</v>
+      </c>
+      <c r="H75" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>311</v>
+      </c>
+      <c r="B76" t="s">
+        <v>17</v>
+      </c>
+      <c r="C76" t="s">
+        <v>312</v>
+      </c>
+      <c r="D76" t="s">
+        <v>11</v>
+      </c>
+      <c r="E76" t="s">
+        <v>19</v>
+      </c>
+      <c r="F76" t="s">
+        <v>313</v>
+      </c>
+      <c r="G76" t="s">
+        <v>21</v>
+      </c>
+      <c r="H76" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>315</v>
+      </c>
+      <c r="B77" t="s">
+        <v>17</v>
+      </c>
+      <c r="C77" t="s">
+        <v>316</v>
+      </c>
+      <c r="D77" t="s">
+        <v>11</v>
+      </c>
+      <c r="E77" t="s">
+        <v>19</v>
+      </c>
+      <c r="F77" t="s">
+        <v>317</v>
+      </c>
+      <c r="G77" t="s">
+        <v>21</v>
+      </c>
+      <c r="H77" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>319</v>
+      </c>
+      <c r="B78" t="s">
+        <v>17</v>
+      </c>
+      <c r="C78" t="s">
+        <v>320</v>
+      </c>
+      <c r="D78" t="s">
+        <v>11</v>
+      </c>
+      <c r="E78" t="s">
+        <v>19</v>
+      </c>
+      <c r="F78" t="s">
+        <v>321</v>
+      </c>
+      <c r="G78" t="s">
+        <v>21</v>
+      </c>
+      <c r="H78" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>323</v>
+      </c>
+      <c r="B79" t="s">
+        <v>17</v>
+      </c>
+      <c r="C79" t="s">
+        <v>324</v>
+      </c>
+      <c r="D79" t="s">
+        <v>11</v>
+      </c>
+      <c r="E79" t="s">
+        <v>19</v>
+      </c>
+      <c r="F79" t="s">
+        <v>325</v>
+      </c>
+      <c r="G79" t="s">
+        <v>21</v>
+      </c>
+      <c r="H79" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>327</v>
+      </c>
+      <c r="B80" t="s">
+        <v>17</v>
+      </c>
+      <c r="C80" t="s">
+        <v>328</v>
+      </c>
+      <c r="D80" t="s">
+        <v>11</v>
+      </c>
+      <c r="E80" t="s">
+        <v>19</v>
+      </c>
+      <c r="F80" t="s">
+        <v>329</v>
+      </c>
+      <c r="G80" t="s">
+        <v>21</v>
+      </c>
+      <c r="H80" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>331</v>
+      </c>
+      <c r="B81" t="s">
+        <v>17</v>
+      </c>
+      <c r="C81" t="s">
+        <v>332</v>
+      </c>
+      <c r="D81" t="s">
+        <v>11</v>
+      </c>
+      <c r="E81" t="s">
+        <v>19</v>
+      </c>
+      <c r="F81" t="s">
+        <v>333</v>
+      </c>
+      <c r="G81" t="s">
+        <v>21</v>
+      </c>
+      <c r="H81" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>335</v>
+      </c>
+      <c r="B82" t="s">
+        <v>17</v>
+      </c>
+      <c r="C82" t="s">
+        <v>336</v>
+      </c>
+      <c r="D82" t="s">
+        <v>11</v>
+      </c>
+      <c r="E82" t="s">
+        <v>19</v>
+      </c>
+      <c r="F82" t="s">
+        <v>337</v>
+      </c>
+      <c r="G82" t="s">
+        <v>21</v>
+      </c>
+      <c r="H82" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>339</v>
+      </c>
+      <c r="B83" t="s">
+        <v>17</v>
+      </c>
+      <c r="C83" t="s">
+        <v>340</v>
+      </c>
+      <c r="D83" t="s">
+        <v>11</v>
+      </c>
+      <c r="E83" t="s">
+        <v>19</v>
+      </c>
+      <c r="F83" t="s">
+        <v>341</v>
+      </c>
+      <c r="G83" t="s">
+        <v>21</v>
+      </c>
+      <c r="H83" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>343</v>
+      </c>
+      <c r="B84" t="s">
+        <v>17</v>
+      </c>
+      <c r="C84" t="s">
+        <v>344</v>
+      </c>
+      <c r="D84" t="s">
+        <v>11</v>
+      </c>
+      <c r="E84" t="s">
+        <v>19</v>
+      </c>
+      <c r="F84" t="s">
+        <v>345</v>
+      </c>
+      <c r="G84" t="s">
+        <v>21</v>
+      </c>
+      <c r="H84" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>347</v>
+      </c>
+      <c r="B85" t="s">
+        <v>17</v>
+      </c>
+      <c r="C85" t="s">
+        <v>348</v>
+      </c>
+      <c r="D85" t="s">
+        <v>11</v>
+      </c>
+      <c r="E85" t="s">
+        <v>19</v>
+      </c>
+      <c r="F85" t="s">
+        <v>349</v>
+      </c>
+      <c r="G85" t="s">
+        <v>21</v>
+      </c>
+      <c r="H85" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>351</v>
+      </c>
+      <c r="B86" t="s">
+        <v>17</v>
+      </c>
+      <c r="C86" t="s">
+        <v>352</v>
+      </c>
+      <c r="D86" t="s">
+        <v>11</v>
+      </c>
+      <c r="E86" t="s">
+        <v>19</v>
+      </c>
+      <c r="F86" t="s">
+        <v>353</v>
+      </c>
+      <c r="G86" t="s">
+        <v>21</v>
+      </c>
+      <c r="H86" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>355</v>
+      </c>
+      <c r="B87" t="s">
+        <v>17</v>
+      </c>
+      <c r="C87" t="s">
+        <v>356</v>
+      </c>
+      <c r="D87" t="s">
+        <v>11</v>
+      </c>
+      <c r="E87" t="s">
+        <v>19</v>
+      </c>
+      <c r="F87" t="s">
+        <v>357</v>
+      </c>
+      <c r="G87" t="s">
+        <v>21</v>
+      </c>
+      <c r="H87" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>359</v>
+      </c>
+      <c r="B88" t="s">
+        <v>17</v>
+      </c>
+      <c r="C88" t="s">
+        <v>360</v>
+      </c>
+      <c r="D88" t="s">
+        <v>11</v>
+      </c>
+      <c r="E88" t="s">
+        <v>19</v>
+      </c>
+      <c r="F88" t="s">
+        <v>361</v>
+      </c>
+      <c r="G88" t="s">
+        <v>21</v>
+      </c>
+      <c r="H88" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>363</v>
+      </c>
+      <c r="B89" t="s">
+        <v>17</v>
+      </c>
+      <c r="C89" t="s">
+        <v>364</v>
+      </c>
+      <c r="D89" t="s">
+        <v>11</v>
+      </c>
+      <c r="E89" t="s">
+        <v>19</v>
+      </c>
+      <c r="F89" t="s">
+        <v>365</v>
+      </c>
+      <c r="G89" t="s">
+        <v>21</v>
+      </c>
+      <c r="H89" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>367</v>
+      </c>
+      <c r="B90" t="s">
+        <v>17</v>
+      </c>
+      <c r="C90" t="s">
+        <v>368</v>
+      </c>
+      <c r="D90" t="s">
+        <v>11</v>
+      </c>
+      <c r="E90" t="s">
+        <v>19</v>
+      </c>
+      <c r="F90" t="s">
+        <v>369</v>
+      </c>
+      <c r="G90" t="s">
+        <v>21</v>
+      </c>
+      <c r="H90" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>371</v>
+      </c>
+      <c r="B91" t="s">
+        <v>17</v>
+      </c>
+      <c r="C91" t="s">
+        <v>372</v>
+      </c>
+      <c r="D91" t="s">
+        <v>11</v>
+      </c>
+      <c r="E91" t="s">
+        <v>19</v>
+      </c>
+      <c r="F91" t="s">
+        <v>373</v>
+      </c>
+      <c r="G91" t="s">
+        <v>21</v>
+      </c>
+      <c r="H91" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>375</v>
+      </c>
+      <c r="B92" t="s">
+        <v>17</v>
+      </c>
+      <c r="C92" t="s">
+        <v>376</v>
+      </c>
+      <c r="D92" t="s">
+        <v>11</v>
+      </c>
+      <c r="E92" t="s">
+        <v>19</v>
+      </c>
+      <c r="F92" t="s">
+        <v>377</v>
+      </c>
+      <c r="G92" t="s">
+        <v>21</v>
+      </c>
+      <c r="H92" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>379</v>
+      </c>
+      <c r="B93" t="s">
+        <v>17</v>
+      </c>
+      <c r="C93" t="s">
+        <v>380</v>
+      </c>
+      <c r="D93" t="s">
+        <v>11</v>
+      </c>
+      <c r="E93" t="s">
+        <v>19</v>
+      </c>
+      <c r="F93" t="s">
+        <v>381</v>
+      </c>
+      <c r="G93" t="s">
+        <v>21</v>
+      </c>
+      <c r="H93" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>383</v>
+      </c>
+      <c r="B94" t="s">
+        <v>17</v>
+      </c>
+      <c r="C94" t="s">
+        <v>384</v>
+      </c>
+      <c r="D94" t="s">
+        <v>11</v>
+      </c>
+      <c r="E94" t="s">
+        <v>19</v>
+      </c>
+      <c r="F94" t="s">
+        <v>385</v>
+      </c>
+      <c r="G94" t="s">
+        <v>21</v>
+      </c>
+      <c r="H94" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>387</v>
+      </c>
+      <c r="B95" t="s">
+        <v>17</v>
+      </c>
+      <c r="C95" t="s">
+        <v>388</v>
+      </c>
+      <c r="D95" t="s">
+        <v>11</v>
+      </c>
+      <c r="E95" t="s">
+        <v>19</v>
+      </c>
+      <c r="F95" t="s">
+        <v>389</v>
+      </c>
+      <c r="G95" t="s">
+        <v>21</v>
+      </c>
+      <c r="H95" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>391</v>
+      </c>
+      <c r="B96" t="s">
+        <v>17</v>
+      </c>
+      <c r="C96" t="s">
+        <v>392</v>
+      </c>
+      <c r="D96" t="s">
+        <v>11</v>
+      </c>
+      <c r="E96" t="s">
+        <v>19</v>
+      </c>
+      <c r="F96" t="s">
+        <v>393</v>
+      </c>
+      <c r="G96" t="s">
+        <v>21</v>
+      </c>
+      <c r="H96" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>395</v>
+      </c>
+      <c r="B97" t="s">
+        <v>17</v>
+      </c>
+      <c r="C97" t="s">
+        <v>396</v>
+      </c>
+      <c r="D97" t="s">
+        <v>11</v>
+      </c>
+      <c r="E97" t="s">
+        <v>19</v>
+      </c>
+      <c r="F97" t="s">
+        <v>397</v>
+      </c>
+      <c r="G97" t="s">
+        <v>21</v>
+      </c>
+      <c r="H97" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>399</v>
+      </c>
+      <c r="B98" t="s">
+        <v>17</v>
+      </c>
+      <c r="C98" t="s">
+        <v>400</v>
+      </c>
+      <c r="D98" t="s">
+        <v>11</v>
+      </c>
+      <c r="E98" t="s">
+        <v>19</v>
+      </c>
+      <c r="F98" t="s">
+        <v>401</v>
+      </c>
+      <c r="G98" t="s">
+        <v>21</v>
+      </c>
+      <c r="H98" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>403</v>
+      </c>
+      <c r="B99" t="s">
+        <v>17</v>
+      </c>
+      <c r="C99" t="s">
+        <v>404</v>
+      </c>
+      <c r="D99" t="s">
+        <v>11</v>
+      </c>
+      <c r="E99" t="s">
+        <v>19</v>
+      </c>
+      <c r="F99" t="s">
+        <v>405</v>
+      </c>
+      <c r="G99" t="s">
+        <v>21</v>
+      </c>
+      <c r="H99" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>407</v>
+      </c>
+      <c r="B100" t="s">
+        <v>17</v>
+      </c>
+      <c r="C100" t="s">
+        <v>408</v>
+      </c>
+      <c r="D100" t="s">
+        <v>11</v>
+      </c>
+      <c r="E100" t="s">
+        <v>19</v>
+      </c>
+      <c r="F100" t="s">
+        <v>409</v>
+      </c>
+      <c r="G100" t="s">
+        <v>21</v>
+      </c>
+      <c r="H100" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>411</v>
+      </c>
+      <c r="B101" t="s">
+        <v>17</v>
+      </c>
+      <c r="C101" t="s">
+        <v>412</v>
+      </c>
+      <c r="D101" t="s">
+        <v>11</v>
+      </c>
+      <c r="E101" t="s">
+        <v>19</v>
+      </c>
+      <c r="F101" t="s">
+        <v>413</v>
+      </c>
+      <c r="G101" t="s">
+        <v>21</v>
+      </c>
+      <c r="H101" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>415</v>
+      </c>
+      <c r="B102" t="s">
+        <v>17</v>
+      </c>
+      <c r="C102" t="s">
+        <v>416</v>
+      </c>
+      <c r="D102" t="s">
+        <v>11</v>
+      </c>
+      <c r="E102" t="s">
+        <v>19</v>
+      </c>
+      <c r="F102" t="s">
+        <v>417</v>
+      </c>
+      <c r="G102" t="s">
+        <v>21</v>
+      </c>
+      <c r="H102" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>419</v>
+      </c>
+      <c r="B103" t="s">
+        <v>17</v>
+      </c>
+      <c r="C103" t="s">
+        <v>420</v>
+      </c>
+      <c r="D103" t="s">
+        <v>11</v>
+      </c>
+      <c r="E103" t="s">
+        <v>19</v>
+      </c>
+      <c r="F103" t="s">
+        <v>421</v>
+      </c>
+      <c r="G103" t="s">
+        <v>21</v>
+      </c>
+      <c r="H103" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>423</v>
+      </c>
+      <c r="B104" t="s">
+        <v>17</v>
+      </c>
+      <c r="C104" t="s">
+        <v>424</v>
+      </c>
+      <c r="D104" t="s">
+        <v>11</v>
+      </c>
+      <c r="E104" t="s">
+        <v>19</v>
+      </c>
+      <c r="F104" t="s">
+        <v>425</v>
+      </c>
+      <c r="G104" t="s">
+        <v>21</v>
+      </c>
+      <c r="H104" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>427</v>
+      </c>
+      <c r="B105" t="s">
+        <v>17</v>
+      </c>
+      <c r="C105" t="s">
+        <v>428</v>
+      </c>
+      <c r="D105" t="s">
+        <v>11</v>
+      </c>
+      <c r="E105" t="s">
+        <v>19</v>
+      </c>
+      <c r="F105" t="s">
+        <v>429</v>
+      </c>
+      <c r="G105" t="s">
+        <v>21</v>
+      </c>
+      <c r="H105" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>431</v>
+      </c>
+      <c r="B106" t="s">
+        <v>17</v>
+      </c>
+      <c r="C106" t="s">
+        <v>432</v>
+      </c>
+      <c r="D106" t="s">
+        <v>11</v>
+      </c>
+      <c r="E106" t="s">
+        <v>19</v>
+      </c>
+      <c r="F106" t="s">
+        <v>433</v>
+      </c>
+      <c r="G106" t="s">
+        <v>21</v>
+      </c>
+      <c r="H106" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>435</v>
+      </c>
+      <c r="B107" t="s">
+        <v>17</v>
+      </c>
+      <c r="C107" t="s">
+        <v>436</v>
+      </c>
+      <c r="D107" t="s">
+        <v>11</v>
+      </c>
+      <c r="E107" t="s">
+        <v>19</v>
+      </c>
+      <c r="F107" t="s">
+        <v>437</v>
+      </c>
+      <c r="G107" t="s">
+        <v>21</v>
+      </c>
+      <c r="H107" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>439</v>
+      </c>
+      <c r="B108" t="s">
+        <v>17</v>
+      </c>
+      <c r="C108" t="s">
+        <v>440</v>
+      </c>
+      <c r="D108" t="s">
+        <v>11</v>
+      </c>
+      <c r="E108" t="s">
+        <v>19</v>
+      </c>
+      <c r="F108" t="s">
+        <v>441</v>
+      </c>
+      <c r="G108" t="s">
+        <v>21</v>
+      </c>
+      <c r="H108" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>443</v>
+      </c>
+      <c r="B109" t="s">
+        <v>17</v>
+      </c>
+      <c r="C109" t="s">
+        <v>444</v>
+      </c>
+      <c r="D109" t="s">
+        <v>11</v>
+      </c>
+      <c r="E109" t="s">
+        <v>19</v>
+      </c>
+      <c r="F109" t="s">
+        <v>445</v>
+      </c>
+      <c r="G109" t="s">
+        <v>21</v>
+      </c>
+      <c r="H109" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>447</v>
+      </c>
+      <c r="B110" t="s">
+        <v>17</v>
+      </c>
+      <c r="C110" t="s">
+        <v>448</v>
+      </c>
+      <c r="D110" t="s">
+        <v>11</v>
+      </c>
+      <c r="E110" t="s">
+        <v>19</v>
+      </c>
+      <c r="F110" t="s">
+        <v>449</v>
+      </c>
+      <c r="G110" t="s">
+        <v>21</v>
+      </c>
+      <c r="H110" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>451</v>
+      </c>
+      <c r="B111" t="s">
+        <v>17</v>
+      </c>
+      <c r="C111" t="s">
+        <v>452</v>
+      </c>
+      <c r="D111" t="s">
+        <v>11</v>
+      </c>
+      <c r="E111" t="s">
+        <v>19</v>
+      </c>
+      <c r="F111" t="s">
+        <v>453</v>
+      </c>
+      <c r="G111" t="s">
+        <v>21</v>
+      </c>
+      <c r="H111" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>455</v>
+      </c>
+      <c r="B112" t="s">
+        <v>17</v>
+      </c>
+      <c r="C112" t="s">
+        <v>456</v>
+      </c>
+      <c r="D112" t="s">
+        <v>11</v>
+      </c>
+      <c r="E112" t="s">
+        <v>19</v>
+      </c>
+      <c r="F112" t="s">
+        <v>457</v>
+      </c>
+      <c r="G112" t="s">
+        <v>21</v>
+      </c>
+      <c r="H112" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>459</v>
+      </c>
+      <c r="B113" t="s">
+        <v>17</v>
+      </c>
+      <c r="C113" t="s">
+        <v>460</v>
+      </c>
+      <c r="D113" t="s">
+        <v>11</v>
+      </c>
+      <c r="E113" t="s">
+        <v>19</v>
+      </c>
+      <c r="F113" t="s">
+        <v>461</v>
+      </c>
+      <c r="G113" t="s">
+        <v>21</v>
+      </c>
+      <c r="H113" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>463</v>
+      </c>
+      <c r="B114" t="s">
+        <v>17</v>
+      </c>
+      <c r="C114" t="s">
+        <v>464</v>
+      </c>
+      <c r="D114" t="s">
+        <v>11</v>
+      </c>
+      <c r="E114" t="s">
+        <v>19</v>
+      </c>
+      <c r="F114" t="s">
+        <v>465</v>
+      </c>
+      <c r="G114" t="s">
+        <v>21</v>
+      </c>
+      <c r="H114" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>467</v>
+      </c>
+      <c r="B115" t="s">
+        <v>17</v>
+      </c>
+      <c r="C115" t="s">
+        <v>468</v>
+      </c>
+      <c r="D115" t="s">
+        <v>11</v>
+      </c>
+      <c r="E115" t="s">
+        <v>19</v>
+      </c>
+      <c r="F115" t="s">
+        <v>469</v>
+      </c>
+      <c r="G115" t="s">
+        <v>21</v>
+      </c>
+      <c r="H115" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>471</v>
+      </c>
+      <c r="B116" t="s">
+        <v>17</v>
+      </c>
+      <c r="C116" t="s">
+        <v>472</v>
+      </c>
+      <c r="D116" t="s">
+        <v>11</v>
+      </c>
+      <c r="E116" t="s">
+        <v>19</v>
+      </c>
+      <c r="F116" t="s">
+        <v>473</v>
+      </c>
+      <c r="G116" t="s">
+        <v>21</v>
+      </c>
+      <c r="H116" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>475</v>
+      </c>
+      <c r="B117" t="s">
+        <v>17</v>
+      </c>
+      <c r="C117" t="s">
+        <v>476</v>
+      </c>
+      <c r="D117" t="s">
+        <v>11</v>
+      </c>
+      <c r="E117" t="s">
+        <v>19</v>
+      </c>
+      <c r="F117" t="s">
+        <v>477</v>
+      </c>
+      <c r="G117" t="s">
+        <v>21</v>
+      </c>
+      <c r="H117" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>479</v>
+      </c>
+      <c r="B118" t="s">
+        <v>17</v>
+      </c>
+      <c r="C118" t="s">
+        <v>480</v>
+      </c>
+      <c r="D118" t="s">
+        <v>11</v>
+      </c>
+      <c r="E118" t="s">
+        <v>19</v>
+      </c>
+      <c r="F118" t="s">
+        <v>481</v>
+      </c>
+      <c r="G118" t="s">
+        <v>21</v>
+      </c>
+      <c r="H118" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>483</v>
+      </c>
+      <c r="B119" t="s">
+        <v>17</v>
+      </c>
+      <c r="C119" t="s">
+        <v>484</v>
+      </c>
+      <c r="D119" t="s">
+        <v>11</v>
+      </c>
+      <c r="E119" t="s">
+        <v>19</v>
+      </c>
+      <c r="F119" t="s">
+        <v>485</v>
+      </c>
+      <c r="G119" t="s">
+        <v>21</v>
+      </c>
+      <c r="H119" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>487</v>
+      </c>
+      <c r="B120" t="s">
+        <v>17</v>
+      </c>
+      <c r="C120" t="s">
+        <v>488</v>
+      </c>
+      <c r="D120" t="s">
+        <v>11</v>
+      </c>
+      <c r="E120" t="s">
+        <v>19</v>
+      </c>
+      <c r="F120" t="s">
+        <v>489</v>
+      </c>
+      <c r="G120" t="s">
+        <v>21</v>
+      </c>
+      <c r="H120" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>491</v>
+      </c>
+      <c r="B121" t="s">
+        <v>17</v>
+      </c>
+      <c r="C121" t="s">
+        <v>492</v>
+      </c>
+      <c r="D121" t="s">
+        <v>11</v>
+      </c>
+      <c r="E121" t="s">
+        <v>19</v>
+      </c>
+      <c r="F121" t="s">
+        <v>493</v>
+      </c>
+      <c r="G121" t="s">
+        <v>21</v>
+      </c>
+      <c r="H121" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>495</v>
+      </c>
+      <c r="B122" t="s">
+        <v>17</v>
+      </c>
+      <c r="C122" t="s">
+        <v>496</v>
+      </c>
+      <c r="D122" t="s">
+        <v>11</v>
+      </c>
+      <c r="E122" t="s">
+        <v>19</v>
+      </c>
+      <c r="F122" t="s">
+        <v>497</v>
+      </c>
+      <c r="G122" t="s">
+        <v>21</v>
+      </c>
+      <c r="H122" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>499</v>
+      </c>
+      <c r="B123" t="s">
+        <v>17</v>
+      </c>
+      <c r="C123" t="s">
+        <v>500</v>
+      </c>
+      <c r="D123" t="s">
+        <v>11</v>
+      </c>
+      <c r="E123" t="s">
+        <v>19</v>
+      </c>
+      <c r="F123" t="s">
+        <v>501</v>
+      </c>
+      <c r="G123" t="s">
+        <v>21</v>
+      </c>
+      <c r="H123" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>503</v>
+      </c>
+      <c r="B124" t="s">
+        <v>17</v>
+      </c>
+      <c r="C124" t="s">
+        <v>504</v>
+      </c>
+      <c r="D124" t="s">
+        <v>11</v>
+      </c>
+      <c r="E124" t="s">
+        <v>19</v>
+      </c>
+      <c r="F124" t="s">
+        <v>505</v>
+      </c>
+      <c r="G124" t="s">
+        <v>21</v>
+      </c>
+      <c r="H124" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>507</v>
+      </c>
+      <c r="B125" t="s">
+        <v>17</v>
+      </c>
+      <c r="C125" t="s">
+        <v>508</v>
+      </c>
+      <c r="D125" t="s">
+        <v>11</v>
+      </c>
+      <c r="E125" t="s">
+        <v>19</v>
+      </c>
+      <c r="F125" t="s">
+        <v>509</v>
+      </c>
+      <c r="G125" t="s">
+        <v>21</v>
+      </c>
+      <c r="H125" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>511</v>
+      </c>
+      <c r="B126" t="s">
+        <v>17</v>
+      </c>
+      <c r="C126" t="s">
+        <v>512</v>
+      </c>
+      <c r="D126" t="s">
+        <v>11</v>
+      </c>
+      <c r="E126" t="s">
+        <v>19</v>
+      </c>
+      <c r="F126" t="s">
+        <v>513</v>
+      </c>
+      <c r="G126" t="s">
+        <v>21</v>
+      </c>
+      <c r="H126" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>515</v>
+      </c>
+      <c r="B127" t="s">
+        <v>17</v>
+      </c>
+      <c r="C127" t="s">
+        <v>516</v>
+      </c>
+      <c r="D127" t="s">
+        <v>11</v>
+      </c>
+      <c r="E127" t="s">
+        <v>19</v>
+      </c>
+      <c r="F127" t="s">
+        <v>517</v>
+      </c>
+      <c r="G127" t="s">
+        <v>21</v>
+      </c>
+      <c r="H127" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>519</v>
+      </c>
+      <c r="B128" t="s">
+        <v>17</v>
+      </c>
+      <c r="C128" t="s">
+        <v>520</v>
+      </c>
+      <c r="D128" t="s">
+        <v>11</v>
+      </c>
+      <c r="E128" t="s">
+        <v>19</v>
+      </c>
+      <c r="F128" t="s">
+        <v>521</v>
+      </c>
+      <c r="G128" t="s">
+        <v>21</v>
+      </c>
+      <c r="H128" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>523</v>
+      </c>
+      <c r="B129" t="s">
+        <v>17</v>
+      </c>
+      <c r="C129" t="s">
+        <v>524</v>
+      </c>
+      <c r="D129" t="s">
+        <v>11</v>
+      </c>
+      <c r="E129" t="s">
+        <v>19</v>
+      </c>
+      <c r="F129" t="s">
+        <v>525</v>
+      </c>
+      <c r="G129" t="s">
+        <v>21</v>
+      </c>
+      <c r="H129" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>527</v>
+      </c>
+      <c r="B130" t="s">
+        <v>17</v>
+      </c>
+      <c r="C130" t="s">
+        <v>528</v>
+      </c>
+      <c r="D130" t="s">
+        <v>11</v>
+      </c>
+      <c r="E130" t="s">
+        <v>19</v>
+      </c>
+      <c r="F130" t="s">
+        <v>529</v>
+      </c>
+      <c r="G130" t="s">
+        <v>21</v>
+      </c>
+      <c r="H130" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>531</v>
+      </c>
+      <c r="B131" t="s">
+        <v>17</v>
+      </c>
+      <c r="C131" t="s">
+        <v>532</v>
+      </c>
+      <c r="D131" t="s">
+        <v>11</v>
+      </c>
+      <c r="E131" t="s">
+        <v>19</v>
+      </c>
+      <c r="F131" t="s">
+        <v>533</v>
+      </c>
+      <c r="G131" t="s">
+        <v>21</v>
+      </c>
+      <c r="H131" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>535</v>
+      </c>
+      <c r="B132" t="s">
+        <v>17</v>
+      </c>
+      <c r="C132" t="s">
+        <v>536</v>
+      </c>
+      <c r="D132" t="s">
+        <v>11</v>
+      </c>
+      <c r="E132" t="s">
+        <v>19</v>
+      </c>
+      <c r="F132" t="s">
+        <v>537</v>
+      </c>
+      <c r="G132" t="s">
+        <v>21</v>
+      </c>
+      <c r="H132" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>539</v>
+      </c>
+      <c r="B133" t="s">
+        <v>17</v>
+      </c>
+      <c r="C133" t="s">
+        <v>540</v>
+      </c>
+      <c r="D133" t="s">
+        <v>11</v>
+      </c>
+      <c r="E133" t="s">
+        <v>19</v>
+      </c>
+      <c r="F133" t="s">
+        <v>541</v>
+      </c>
+      <c r="G133" t="s">
+        <v>21</v>
+      </c>
+      <c r="H133" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>543</v>
+      </c>
+      <c r="B134" t="s">
+        <v>17</v>
+      </c>
+      <c r="C134" t="s">
+        <v>544</v>
+      </c>
+      <c r="D134" t="s">
+        <v>11</v>
+      </c>
+      <c r="E134" t="s">
+        <v>19</v>
+      </c>
+      <c r="F134" t="s">
+        <v>545</v>
+      </c>
+      <c r="G134" t="s">
+        <v>21</v>
+      </c>
+      <c r="H134" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>547</v>
+      </c>
+      <c r="B135" t="s">
+        <v>17</v>
+      </c>
+      <c r="C135" t="s">
+        <v>548</v>
+      </c>
+      <c r="D135" t="s">
+        <v>11</v>
+      </c>
+      <c r="E135" t="s">
+        <v>19</v>
+      </c>
+      <c r="F135" t="s">
+        <v>549</v>
+      </c>
+      <c r="G135" t="s">
+        <v>21</v>
+      </c>
+      <c r="H135" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>551</v>
+      </c>
+      <c r="B136" t="s">
+        <v>17</v>
+      </c>
+      <c r="C136" t="s">
+        <v>552</v>
+      </c>
+      <c r="D136" t="s">
+        <v>11</v>
+      </c>
+      <c r="E136" t="s">
+        <v>19</v>
+      </c>
+      <c r="F136" t="s">
+        <v>553</v>
+      </c>
+      <c r="G136" t="s">
+        <v>21</v>
+      </c>
+      <c r="H136" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>555</v>
+      </c>
+      <c r="B137" t="s">
+        <v>17</v>
+      </c>
+      <c r="C137" t="s">
+        <v>556</v>
+      </c>
+      <c r="D137" t="s">
+        <v>11</v>
+      </c>
+      <c r="E137" t="s">
+        <v>19</v>
+      </c>
+      <c r="F137" t="s">
+        <v>557</v>
+      </c>
+      <c r="G137" t="s">
+        <v>21</v>
+      </c>
+      <c r="H137" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>559</v>
+      </c>
+      <c r="B138" t="s">
+        <v>17</v>
+      </c>
+      <c r="C138" t="s">
+        <v>560</v>
+      </c>
+      <c r="D138" t="s">
+        <v>11</v>
+      </c>
+      <c r="E138" t="s">
+        <v>19</v>
+      </c>
+      <c r="F138" t="s">
+        <v>561</v>
+      </c>
+      <c r="G138" t="s">
+        <v>21</v>
+      </c>
+      <c r="H138" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>563</v>
+      </c>
+      <c r="B139" t="s">
+        <v>17</v>
+      </c>
+      <c r="C139" t="s">
+        <v>564</v>
+      </c>
+      <c r="D139" t="s">
+        <v>11</v>
+      </c>
+      <c r="E139" t="s">
+        <v>19</v>
+      </c>
+      <c r="F139" t="s">
+        <v>565</v>
+      </c>
+      <c r="G139" t="s">
+        <v>21</v>
+      </c>
+      <c r="H139" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>567</v>
+      </c>
+      <c r="B140" t="s">
+        <v>17</v>
+      </c>
+      <c r="C140" t="s">
+        <v>568</v>
+      </c>
+      <c r="D140" t="s">
+        <v>11</v>
+      </c>
+      <c r="E140" t="s">
+        <v>19</v>
+      </c>
+      <c r="F140" t="s">
+        <v>569</v>
+      </c>
+      <c r="G140" t="s">
+        <v>21</v>
+      </c>
+      <c r="H140" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>571</v>
+      </c>
+      <c r="B141" t="s">
+        <v>17</v>
+      </c>
+      <c r="C141" t="s">
+        <v>572</v>
+      </c>
+      <c r="D141" t="s">
+        <v>11</v>
+      </c>
+      <c r="E141" t="s">
+        <v>19</v>
+      </c>
+      <c r="F141" t="s">
+        <v>573</v>
+      </c>
+      <c r="G141" t="s">
+        <v>21</v>
+      </c>
+      <c r="H141" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>575</v>
+      </c>
+      <c r="B142" t="s">
+        <v>17</v>
+      </c>
+      <c r="C142" t="s">
+        <v>576</v>
+      </c>
+      <c r="D142" t="s">
+        <v>11</v>
+      </c>
+      <c r="E142" t="s">
+        <v>19</v>
+      </c>
+      <c r="F142" t="s">
+        <v>577</v>
+      </c>
+      <c r="G142" t="s">
+        <v>21</v>
+      </c>
+      <c r="H142" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>579</v>
+      </c>
+      <c r="B143" t="s">
+        <v>17</v>
+      </c>
+      <c r="C143" t="s">
+        <v>580</v>
+      </c>
+      <c r="D143" t="s">
+        <v>11</v>
+      </c>
+      <c r="E143" t="s">
+        <v>19</v>
+      </c>
+      <c r="F143" t="s">
+        <v>581</v>
+      </c>
+      <c r="G143" t="s">
+        <v>21</v>
+      </c>
+      <c r="H143" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>583</v>
+      </c>
+      <c r="B144" t="s">
+        <v>17</v>
+      </c>
+      <c r="C144" t="s">
+        <v>584</v>
+      </c>
+      <c r="D144" t="s">
+        <v>11</v>
+      </c>
+      <c r="E144" t="s">
+        <v>19</v>
+      </c>
+      <c r="F144" t="s">
+        <v>585</v>
+      </c>
+      <c r="G144" t="s">
+        <v>21</v>
+      </c>
+      <c r="H144" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>587</v>
+      </c>
+      <c r="B145" t="s">
+        <v>17</v>
+      </c>
+      <c r="C145" t="s">
+        <v>588</v>
+      </c>
+      <c r="D145" t="s">
+        <v>11</v>
+      </c>
+      <c r="E145" t="s">
+        <v>19</v>
+      </c>
+      <c r="F145" t="s">
+        <v>589</v>
+      </c>
+      <c r="G145" t="s">
+        <v>21</v>
+      </c>
+      <c r="H145" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>591</v>
+      </c>
+      <c r="B146" t="s">
+        <v>17</v>
+      </c>
+      <c r="C146" t="s">
+        <v>592</v>
+      </c>
+      <c r="D146" t="s">
+        <v>11</v>
+      </c>
+      <c r="E146" t="s">
+        <v>19</v>
+      </c>
+      <c r="F146" t="s">
+        <v>593</v>
+      </c>
+      <c r="G146" t="s">
+        <v>21</v>
+      </c>
+      <c r="H146" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>595</v>
+      </c>
+      <c r="B147" t="s">
+        <v>17</v>
+      </c>
+      <c r="C147" t="s">
+        <v>596</v>
+      </c>
+      <c r="D147" t="s">
+        <v>11</v>
+      </c>
+      <c r="E147" t="s">
+        <v>19</v>
+      </c>
+      <c r="F147" t="s">
+        <v>597</v>
+      </c>
+      <c r="G147" t="s">
+        <v>21</v>
+      </c>
+      <c r="H147" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>599</v>
+      </c>
+      <c r="B148" t="s">
+        <v>17</v>
+      </c>
+      <c r="C148" t="s">
+        <v>600</v>
+      </c>
+      <c r="D148" t="s">
+        <v>11</v>
+      </c>
+      <c r="E148" t="s">
+        <v>19</v>
+      </c>
+      <c r="F148" t="s">
+        <v>601</v>
+      </c>
+      <c r="G148" t="s">
+        <v>21</v>
+      </c>
+      <c r="H148" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>603</v>
+      </c>
+      <c r="B149" t="s">
+        <v>17</v>
+      </c>
+      <c r="C149" t="s">
+        <v>604</v>
+      </c>
+      <c r="D149" t="s">
+        <v>11</v>
+      </c>
+      <c r="E149" t="s">
+        <v>19</v>
+      </c>
+      <c r="F149" t="s">
+        <v>605</v>
+      </c>
+      <c r="G149" t="s">
+        <v>21</v>
+      </c>
+      <c r="H149" t="s">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>607</v>
+      </c>
+      <c r="B150" t="s">
+        <v>17</v>
+      </c>
+      <c r="C150" t="s">
+        <v>608</v>
+      </c>
+      <c r="D150" t="s">
+        <v>11</v>
+      </c>
+      <c r="E150" t="s">
+        <v>19</v>
+      </c>
+      <c r="F150" t="s">
+        <v>609</v>
+      </c>
+      <c r="G150" t="s">
+        <v>21</v>
+      </c>
+      <c r="H150" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>611</v>
+      </c>
+      <c r="B151" t="s">
+        <v>17</v>
+      </c>
+      <c r="C151" t="s">
+        <v>612</v>
+      </c>
+      <c r="D151" t="s">
+        <v>11</v>
+      </c>
+      <c r="E151" t="s">
+        <v>19</v>
+      </c>
+      <c r="F151" t="s">
+        <v>613</v>
+      </c>
+      <c r="G151" t="s">
+        <v>21</v>
+      </c>
+      <c r="H151" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>615</v>
+      </c>
+      <c r="B152" t="s">
+        <v>17</v>
+      </c>
+      <c r="C152" t="s">
+        <v>616</v>
+      </c>
+      <c r="D152" t="s">
+        <v>11</v>
+      </c>
+      <c r="E152" t="s">
+        <v>19</v>
+      </c>
+      <c r="F152" t="s">
+        <v>617</v>
+      </c>
+      <c r="G152" t="s">
+        <v>21</v>
+      </c>
+      <c r="H152" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>619</v>
+      </c>
+      <c r="B153" t="s">
+        <v>17</v>
+      </c>
+      <c r="C153" t="s">
+        <v>620</v>
+      </c>
+      <c r="D153" t="s">
+        <v>11</v>
+      </c>
+      <c r="E153" t="s">
+        <v>19</v>
+      </c>
+      <c r="F153" t="s">
+        <v>621</v>
+      </c>
+      <c r="G153" t="s">
+        <v>21</v>
+      </c>
+      <c r="H153" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>623</v>
+      </c>
+      <c r="B154" t="s">
+        <v>17</v>
+      </c>
+      <c r="C154" t="s">
+        <v>624</v>
+      </c>
+      <c r="D154" t="s">
+        <v>11</v>
+      </c>
+      <c r="E154" t="s">
+        <v>19</v>
+      </c>
+      <c r="F154" t="s">
+        <v>625</v>
+      </c>
+      <c r="G154" t="s">
+        <v>21</v>
+      </c>
+      <c r="H154" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>627</v>
+      </c>
+      <c r="B155" t="s">
+        <v>17</v>
+      </c>
+      <c r="C155" t="s">
+        <v>628</v>
+      </c>
+      <c r="D155" t="s">
+        <v>11</v>
+      </c>
+      <c r="E155" t="s">
+        <v>19</v>
+      </c>
+      <c r="F155" t="s">
+        <v>629</v>
+      </c>
+      <c r="G155" t="s">
+        <v>21</v>
+      </c>
+      <c r="H155" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>631</v>
+      </c>
+      <c r="B156" t="s">
+        <v>17</v>
+      </c>
+      <c r="C156" t="s">
+        <v>632</v>
+      </c>
+      <c r="D156" t="s">
+        <v>11</v>
+      </c>
+      <c r="E156" t="s">
+        <v>19</v>
+      </c>
+      <c r="F156" t="s">
+        <v>633</v>
+      </c>
+      <c r="G156" t="s">
+        <v>21</v>
+      </c>
+      <c r="H156" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>635</v>
+      </c>
+      <c r="B157" t="s">
+        <v>17</v>
+      </c>
+      <c r="C157" t="s">
+        <v>636</v>
+      </c>
+      <c r="D157" t="s">
+        <v>11</v>
+      </c>
+      <c r="E157" t="s">
+        <v>19</v>
+      </c>
+      <c r="F157" t="s">
+        <v>637</v>
+      </c>
+      <c r="G157" t="s">
+        <v>21</v>
+      </c>
+      <c r="H157" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>639</v>
+      </c>
+      <c r="B158" t="s">
+        <v>17</v>
+      </c>
+      <c r="C158" t="s">
+        <v>640</v>
+      </c>
+      <c r="D158" t="s">
+        <v>11</v>
+      </c>
+      <c r="E158" t="s">
+        <v>19</v>
+      </c>
+      <c r="F158" t="s">
+        <v>641</v>
+      </c>
+      <c r="G158" t="s">
+        <v>21</v>
+      </c>
+      <c r="H158" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>643</v>
+      </c>
+      <c r="B159" t="s">
+        <v>17</v>
+      </c>
+      <c r="C159" t="s">
+        <v>644</v>
+      </c>
+      <c r="D159" t="s">
+        <v>11</v>
+      </c>
+      <c r="E159" t="s">
+        <v>19</v>
+      </c>
+      <c r="F159" t="s">
+        <v>645</v>
+      </c>
+      <c r="G159" t="s">
+        <v>21</v>
+      </c>
+      <c r="H159" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>647</v>
+      </c>
+      <c r="B160" t="s">
+        <v>17</v>
+      </c>
+      <c r="C160" t="s">
+        <v>648</v>
+      </c>
+      <c r="D160" t="s">
+        <v>11</v>
+      </c>
+      <c r="E160" t="s">
+        <v>19</v>
+      </c>
+      <c r="F160" t="s">
+        <v>649</v>
+      </c>
+      <c r="G160" t="s">
+        <v>21</v>
+      </c>
+      <c r="H160" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>651</v>
+      </c>
+      <c r="B161" t="s">
+        <v>17</v>
+      </c>
+      <c r="C161" t="s">
+        <v>652</v>
+      </c>
+      <c r="D161" t="s">
+        <v>11</v>
+      </c>
+      <c r="E161" t="s">
+        <v>19</v>
+      </c>
+      <c r="F161" t="s">
+        <v>653</v>
+      </c>
+      <c r="G161" t="s">
+        <v>21</v>
+      </c>
+      <c r="H161" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>655</v>
+      </c>
+      <c r="B162" t="s">
+        <v>17</v>
+      </c>
+      <c r="C162" t="s">
+        <v>656</v>
+      </c>
+      <c r="D162" t="s">
+        <v>11</v>
+      </c>
+      <c r="E162" t="s">
+        <v>19</v>
+      </c>
+      <c r="F162" t="s">
+        <v>657</v>
+      </c>
+      <c r="G162" t="s">
+        <v>21</v>
+      </c>
+      <c r="H162" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="163" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>659</v>
+      </c>
+      <c r="B163" t="s">
+        <v>17</v>
+      </c>
+      <c r="C163" t="s">
+        <v>660</v>
+      </c>
+      <c r="D163" t="s">
+        <v>11</v>
+      </c>
+      <c r="E163" t="s">
+        <v>19</v>
+      </c>
+      <c r="F163" t="s">
+        <v>661</v>
+      </c>
+      <c r="G163" t="s">
+        <v>21</v>
+      </c>
+      <c r="H163" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="164" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>663</v>
+      </c>
+      <c r="B164" t="s">
+        <v>17</v>
+      </c>
+      <c r="C164" t="s">
+        <v>664</v>
+      </c>
+      <c r="D164" t="s">
+        <v>11</v>
+      </c>
+      <c r="E164" t="s">
+        <v>19</v>
+      </c>
+      <c r="F164" t="s">
+        <v>665</v>
+      </c>
+      <c r="G164" t="s">
+        <v>21</v>
+      </c>
+      <c r="H164" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="165" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>667</v>
+      </c>
+      <c r="B165" t="s">
+        <v>17</v>
+      </c>
+      <c r="C165" t="s">
+        <v>668</v>
+      </c>
+      <c r="D165" t="s">
+        <v>11</v>
+      </c>
+      <c r="E165" t="s">
+        <v>19</v>
+      </c>
+      <c r="F165" t="s">
+        <v>669</v>
+      </c>
+      <c r="G165" t="s">
+        <v>21</v>
+      </c>
+      <c r="H165" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="166" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
+        <v>671</v>
+      </c>
+      <c r="B166" t="s">
+        <v>17</v>
+      </c>
+      <c r="C166" t="s">
+        <v>672</v>
+      </c>
+      <c r="D166" t="s">
+        <v>11</v>
+      </c>
+      <c r="E166" t="s">
+        <v>19</v>
+      </c>
+      <c r="F166" t="s">
+        <v>673</v>
+      </c>
+      <c r="G166" t="s">
+        <v>21</v>
+      </c>
+      <c r="H166" t="s">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="167" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
+        <v>675</v>
+      </c>
+      <c r="B167" t="s">
+        <v>17</v>
+      </c>
+      <c r="C167" t="s">
+        <v>676</v>
+      </c>
+      <c r="D167" t="s">
+        <v>11</v>
+      </c>
+      <c r="E167" t="s">
+        <v>19</v>
+      </c>
+      <c r="F167" t="s">
+        <v>677</v>
+      </c>
+      <c r="G167" t="s">
+        <v>21</v>
+      </c>
+      <c r="H167" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="168" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
+        <v>679</v>
+      </c>
+      <c r="B168" t="s">
+        <v>17</v>
+      </c>
+      <c r="C168" t="s">
+        <v>680</v>
+      </c>
+      <c r="D168" t="s">
+        <v>11</v>
+      </c>
+      <c r="E168" t="s">
+        <v>19</v>
+      </c>
+      <c r="F168" t="s">
+        <v>681</v>
+      </c>
+      <c r="G168" t="s">
+        <v>21</v>
+      </c>
+      <c r="H168" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="169" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
+        <v>683</v>
+      </c>
+      <c r="B169" t="s">
+        <v>17</v>
+      </c>
+      <c r="C169" t="s">
+        <v>684</v>
+      </c>
+      <c r="D169" t="s">
+        <v>11</v>
+      </c>
+      <c r="E169" t="s">
+        <v>19</v>
+      </c>
+      <c r="F169" t="s">
+        <v>685</v>
+      </c>
+      <c r="G169" t="s">
+        <v>21</v>
+      </c>
+      <c r="H169" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="170" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
+        <v>687</v>
+      </c>
+      <c r="B170" t="s">
+        <v>17</v>
+      </c>
+      <c r="C170" t="s">
+        <v>688</v>
+      </c>
+      <c r="D170" t="s">
+        <v>11</v>
+      </c>
+      <c r="E170" t="s">
+        <v>19</v>
+      </c>
+      <c r="F170" t="s">
+        <v>689</v>
+      </c>
+      <c r="G170" t="s">
+        <v>21</v>
+      </c>
+      <c r="H170" t="s">
         <v>86</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Migrate newsroom Facebook Rules page; unwrap archived links
Import /us/en/newsroom/facebook-rules via the existing article template
(identical structure: article-header, hero, body, social-share). Add a
cleanup-transformer rule that unwraps web.archive.org-wrapped hrefs back to
their original destination, so the Facebook Terms and ups.com links point
live instead of at the Wayback Machine.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article.report.xlsx
+++ b/tools/importer/reports/import-article.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1360" uniqueCount="690">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1368" uniqueCount="694">
   <si>
     <t>_reportFile</t>
   </si>
@@ -61,22 +61,34 @@
     <t>https://about.ups.com/us/en/home.html</t>
   </si>
   <si>
+    <t>language-masters/en/newsroom/facebook-rules.report.json</t>
+  </si>
+  <si>
+    <t>["article"]</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/facebook-rules</t>
+  </si>
+  <si>
+    <t>article</t>
+  </si>
+  <si>
+    <t>2026-07-30T09:50:53.485Z</t>
+  </si>
+  <si>
+    <t>Article</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/facebook-rules.html</t>
+  </si>
+  <si>
     <t>language-masters/en/newsroom/press-releases/customer-first/interglobe-enterprises-and-ups-launch-movin.report.json</t>
   </si>
   <si>
-    <t>["article"]</t>
-  </si>
-  <si>
     <t>language-masters/en/newsroom/press-releases/customer-first/interglobe-enterprises-and-ups-launch-movin</t>
   </si>
   <si>
-    <t>article</t>
-  </si>
-  <si>
     <t>2026-07-10T12:27:01.678Z</t>
-  </si>
-  <si>
-    <t>Article</t>
   </si>
   <si>
     <t>https://about.ups.com/us/en/newsroom/press-releases/customer-first/interglobe-enterprises-and-ups-launch-movin-.html</t>
@@ -2469,7 +2481,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H170"/>
+  <dimension ref="A1:H171"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -6896,7 +6908,33 @@
         <v>21</v>
       </c>
       <c r="H170" t="s">
-        <v>86</v>
+        <v>690</v>
+      </c>
+    </row>
+    <row r="171" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>691</v>
+      </c>
+      <c r="B171" t="s">
+        <v>17</v>
+      </c>
+      <c r="C171" t="s">
+        <v>692</v>
+      </c>
+      <c r="D171" t="s">
+        <v>11</v>
+      </c>
+      <c r="E171" t="s">
+        <v>19</v>
+      </c>
+      <c r="F171" t="s">
+        <v>693</v>
+      </c>
+      <c r="G171" t="s">
+        <v>21</v>
+      </c>
+      <c r="H171" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Migrate 14 newsroom statement/negotiation pages via article template
Bulk-import the negotiations ratify page and 13 statements pages using the
customer-first article structure. Fix the article parser to handle bodies
authored as bare text directly inside .cmp-text (no <p> wrapper) — two pages
(aircraft-maintenance, fredrick-w-smith) were importing with empty bodies;
the parser now wraps raw .cmp-text content in a paragraph as a fallback.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article.report.xlsx
+++ b/tools/importer/reports/import-article.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1368" uniqueCount="694">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1480" uniqueCount="750">
   <si>
     <t>_reportFile</t>
   </si>
@@ -80,6 +80,174 @@
   </si>
   <si>
     <t>https://about.ups.com/us/en/newsroom/facebook-rules.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/negotiations/ups-teamsters-vote-to-overwhelming-ratify-national-master-agreem.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/negotiations/ups-teamsters-vote-to-overwhelming-ratify-national-master-agreem</t>
+  </si>
+  <si>
+    <t>2026-07-30T11:27:26.579Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/negotiations/ups-teamsters-vote-to-overwhelming-ratify-national-master-agreem.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/aircraft-maintenance-contract-agreement.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/aircraft-maintenance-contract-agreement</t>
+  </si>
+  <si>
+    <t>2026-07-30T11:32:37.004Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/statements/aircraft-maintenance-contract-agreement.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/an-update-on-changes-to-our-u-s-network-operations.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/an-update-on-changes-to-our-u-s-network-operations</t>
+  </si>
+  <si>
+    <t>2026-07-30T11:27:37.022Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/statements/an-update-on-changes-to-our-u-s--network-operations-.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/statement-from-carol-tome-on-kevin-warsh-nomination.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/statement-from-carol-tome-on-kevin-warsh-nomination</t>
+  </si>
+  <si>
+    <t>2026-07-30T11:27:42.471Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/statements/statement-from-carol-tome-on-kevin-warsh-nomination.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/statement-from-ups-on-the-passing-of-president-jimmy-carter.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/statement-from-ups-on-the-passing-of-president-jimmy-carter</t>
+  </si>
+  <si>
+    <t>2026-07-30T11:27:48.154Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/statements/statement-from-ups-on-the-passing-of-president-jimmy-carter.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/ups-announces-u-s-driver-voluntary-program.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/ups-announces-u-s-driver-voluntary-program</t>
+  </si>
+  <si>
+    <t>2026-07-30T11:27:54.721Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/statements/ups-announces-u-s--driver-voluntary-program.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/ups-reaches-agreement-with-teamsters-on-driver-choice-program.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/ups-reaches-agreement-with-teamsters-on-driver-choice-program</t>
+  </si>
+  <si>
+    <t>2026-07-30T11:28:02.209Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/statements/ups-reaches-agreement-with-teamsters-on-driver-choice-program.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/ups-statement-in-memory-of-fredrick-w-smith.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/ups-statement-in-memory-of-fredrick-w-smith</t>
+  </si>
+  <si>
+    <t>2026-07-30T11:32:43.193Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/statements/ups-statement-in-memory-of-fredrick-w--smith-.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/ups-statement-on-aircraft-accident.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/ups-statement-on-aircraft-accident</t>
+  </si>
+  <si>
+    <t>2026-07-30T11:28:12.123Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/statements/ups-statement-on-aircraft-accident.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/ups-statement-on-md-11-fleet.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/ups-statement-on-md-11-fleet</t>
+  </si>
+  <si>
+    <t>2026-07-30T11:28:17.822Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/statements/ups-statement-on-md-11-fleet.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/ups-statement-on-new-people-investments.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/ups-statement-on-new-people-investments</t>
+  </si>
+  <si>
+    <t>2026-07-30T11:28:23.100Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/statements/ups-statement-on-new-people-investments.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/ups-statement-on-the-passing-of-first-lady-rosalynn-carter.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/ups-statement-on-the-passing-of-first-lady-rosalynn-carter</t>
+  </si>
+  <si>
+    <t>2026-07-30T11:28:29.807Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/statements/ups-statement-on-the-passing-of-first-lady-rosalynn-carter.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/ups-statement-on-u-s-driver-voluntary-program.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/ups-statement-on-u-s-driver-voluntary-program</t>
+  </si>
+  <si>
+    <t>2026-07-30T11:28:34.766Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/statements/ups-statement-on-u-s--driver-voluntary-program.html</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/ups-statement-on-u-s-network-optimization.report.json</t>
+  </si>
+  <si>
+    <t>language-masters/en/newsroom/statements/ups-statement-on-u-s-network-optimization</t>
+  </si>
+  <si>
+    <t>2026-07-30T11:28:40.256Z</t>
+  </si>
+  <si>
+    <t>https://about.ups.com/us/en/newsroom/statements/ups-statement-on-u-s--network-optimization.html</t>
   </si>
   <si>
     <t>language-masters/en/newsroom/press-releases/customer-first/interglobe-enterprises-and-ups-launch-movin.report.json</t>
@@ -2481,7 +2649,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H171"/>
+  <dimension ref="A1:H185"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -6934,7 +7102,371 @@
         <v>21</v>
       </c>
       <c r="H171" t="s">
-        <v>90</v>
+        <v>694</v>
+      </c>
+    </row>
+    <row r="172" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>695</v>
+      </c>
+      <c r="B172" t="s">
+        <v>17</v>
+      </c>
+      <c r="C172" t="s">
+        <v>696</v>
+      </c>
+      <c r="D172" t="s">
+        <v>11</v>
+      </c>
+      <c r="E172" t="s">
+        <v>19</v>
+      </c>
+      <c r="F172" t="s">
+        <v>697</v>
+      </c>
+      <c r="G172" t="s">
+        <v>21</v>
+      </c>
+      <c r="H172" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="173" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>699</v>
+      </c>
+      <c r="B173" t="s">
+        <v>17</v>
+      </c>
+      <c r="C173" t="s">
+        <v>700</v>
+      </c>
+      <c r="D173" t="s">
+        <v>11</v>
+      </c>
+      <c r="E173" t="s">
+        <v>19</v>
+      </c>
+      <c r="F173" t="s">
+        <v>701</v>
+      </c>
+      <c r="G173" t="s">
+        <v>21</v>
+      </c>
+      <c r="H173" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="174" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>703</v>
+      </c>
+      <c r="B174" t="s">
+        <v>17</v>
+      </c>
+      <c r="C174" t="s">
+        <v>704</v>
+      </c>
+      <c r="D174" t="s">
+        <v>11</v>
+      </c>
+      <c r="E174" t="s">
+        <v>19</v>
+      </c>
+      <c r="F174" t="s">
+        <v>705</v>
+      </c>
+      <c r="G174" t="s">
+        <v>21</v>
+      </c>
+      <c r="H174" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="175" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>707</v>
+      </c>
+      <c r="B175" t="s">
+        <v>17</v>
+      </c>
+      <c r="C175" t="s">
+        <v>708</v>
+      </c>
+      <c r="D175" t="s">
+        <v>11</v>
+      </c>
+      <c r="E175" t="s">
+        <v>19</v>
+      </c>
+      <c r="F175" t="s">
+        <v>709</v>
+      </c>
+      <c r="G175" t="s">
+        <v>21</v>
+      </c>
+      <c r="H175" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
+        <v>711</v>
+      </c>
+      <c r="B176" t="s">
+        <v>17</v>
+      </c>
+      <c r="C176" t="s">
+        <v>712</v>
+      </c>
+      <c r="D176" t="s">
+        <v>11</v>
+      </c>
+      <c r="E176" t="s">
+        <v>19</v>
+      </c>
+      <c r="F176" t="s">
+        <v>713</v>
+      </c>
+      <c r="G176" t="s">
+        <v>21</v>
+      </c>
+      <c r="H176" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="177" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>715</v>
+      </c>
+      <c r="B177" t="s">
+        <v>17</v>
+      </c>
+      <c r="C177" t="s">
+        <v>716</v>
+      </c>
+      <c r="D177" t="s">
+        <v>11</v>
+      </c>
+      <c r="E177" t="s">
+        <v>19</v>
+      </c>
+      <c r="F177" t="s">
+        <v>717</v>
+      </c>
+      <c r="G177" t="s">
+        <v>21</v>
+      </c>
+      <c r="H177" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="178" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>719</v>
+      </c>
+      <c r="B178" t="s">
+        <v>17</v>
+      </c>
+      <c r="C178" t="s">
+        <v>720</v>
+      </c>
+      <c r="D178" t="s">
+        <v>11</v>
+      </c>
+      <c r="E178" t="s">
+        <v>19</v>
+      </c>
+      <c r="F178" t="s">
+        <v>721</v>
+      </c>
+      <c r="G178" t="s">
+        <v>21</v>
+      </c>
+      <c r="H178" t="s">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="179" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>723</v>
+      </c>
+      <c r="B179" t="s">
+        <v>17</v>
+      </c>
+      <c r="C179" t="s">
+        <v>724</v>
+      </c>
+      <c r="D179" t="s">
+        <v>11</v>
+      </c>
+      <c r="E179" t="s">
+        <v>19</v>
+      </c>
+      <c r="F179" t="s">
+        <v>725</v>
+      </c>
+      <c r="G179" t="s">
+        <v>21</v>
+      </c>
+      <c r="H179" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="180" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>727</v>
+      </c>
+      <c r="B180" t="s">
+        <v>17</v>
+      </c>
+      <c r="C180" t="s">
+        <v>728</v>
+      </c>
+      <c r="D180" t="s">
+        <v>11</v>
+      </c>
+      <c r="E180" t="s">
+        <v>19</v>
+      </c>
+      <c r="F180" t="s">
+        <v>729</v>
+      </c>
+      <c r="G180" t="s">
+        <v>21</v>
+      </c>
+      <c r="H180" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="181" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>731</v>
+      </c>
+      <c r="B181" t="s">
+        <v>17</v>
+      </c>
+      <c r="C181" t="s">
+        <v>732</v>
+      </c>
+      <c r="D181" t="s">
+        <v>11</v>
+      </c>
+      <c r="E181" t="s">
+        <v>19</v>
+      </c>
+      <c r="F181" t="s">
+        <v>733</v>
+      </c>
+      <c r="G181" t="s">
+        <v>21</v>
+      </c>
+      <c r="H181" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="182" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>735</v>
+      </c>
+      <c r="B182" t="s">
+        <v>17</v>
+      </c>
+      <c r="C182" t="s">
+        <v>736</v>
+      </c>
+      <c r="D182" t="s">
+        <v>11</v>
+      </c>
+      <c r="E182" t="s">
+        <v>19</v>
+      </c>
+      <c r="F182" t="s">
+        <v>737</v>
+      </c>
+      <c r="G182" t="s">
+        <v>21</v>
+      </c>
+      <c r="H182" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="183" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>739</v>
+      </c>
+      <c r="B183" t="s">
+        <v>17</v>
+      </c>
+      <c r="C183" t="s">
+        <v>740</v>
+      </c>
+      <c r="D183" t="s">
+        <v>11</v>
+      </c>
+      <c r="E183" t="s">
+        <v>19</v>
+      </c>
+      <c r="F183" t="s">
+        <v>741</v>
+      </c>
+      <c r="G183" t="s">
+        <v>21</v>
+      </c>
+      <c r="H183" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="184" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>743</v>
+      </c>
+      <c r="B184" t="s">
+        <v>17</v>
+      </c>
+      <c r="C184" t="s">
+        <v>744</v>
+      </c>
+      <c r="D184" t="s">
+        <v>11</v>
+      </c>
+      <c r="E184" t="s">
+        <v>19</v>
+      </c>
+      <c r="F184" t="s">
+        <v>745</v>
+      </c>
+      <c r="G184" t="s">
+        <v>21</v>
+      </c>
+      <c r="H184" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="185" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
+        <v>747</v>
+      </c>
+      <c r="B185" t="s">
+        <v>17</v>
+      </c>
+      <c r="C185" t="s">
+        <v>748</v>
+      </c>
+      <c r="D185" t="s">
+        <v>11</v>
+      </c>
+      <c r="E185" t="s">
+        <v>19</v>
+      </c>
+      <c r="F185" t="s">
+        <v>749</v>
+      </c>
+      <c r="G185" t="s">
+        <v>21</v>
+      </c>
+      <c r="H185" t="s">
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>